<commit_message>
Update soccer trades 2026-07-30 13:02:57 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/First League/trades.xlsx
+++ b/data/sxbet/ligas/First League/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,110 +531,214 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>0x4449ee9e19610ed1a6459a4ec622295d3b7f27785ad56fb418383aa2562ee601</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0x34FcBC23fB24111d68542f4B3cF185543Af2fA25</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.5987</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>First League</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>FK Pardubice vs FK Jablonec</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>FK Pardubice</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>FK Jablonec</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0x6f33961a8aeffc315ff5d4a74c7a39f6142a8a7935508f048474d0ff32992a6d</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>L19527406</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>1785415503</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1785693600</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>58.455115</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>0x19f2092f5b69321f498e3935667243b7f359a9876c356076e23b9a65276c6308</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>0.99998</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>1.8363</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>AC Sparta Praha</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>First League</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>AC Sparta Praha vs FC Fastav Zlín</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>AC Sparta Praha</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>FC Fastav Zlín</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>0x030b420c1d99e5824e84934cc2cf515e30fa8607adbe9c86574bc07d04d89b58</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>L19527404</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>1785344291</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>1785517200</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>1.195791</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-31 05:02:57 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/First League/trades.xlsx
+++ b/data/sxbet/ligas/First League/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,23 +531,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x4449ee9e19610ed1a6459a4ec622295d3b7f27785ad56fb418383aa2562ee601</t>
+          <t>0x5743b3baab7d0b4196ffe72f2ea5f72938b9bc8bd6e7156319c249a8e1d4977e</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x34FcBC23fB24111d68542f4B3cF185543Af2fA25</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5987</t>
+          <t>1.0625</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,7 +559,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>First League</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>FK Pardubice vs FK Jablonec</t>
+          <t>AC Sparta Praha vs FC Fastav Zlín</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>FK Pardubice</t>
+          <t>AC Sparta Praha</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>FK Jablonec</t>
+          <t>FC Fastav Zlín</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x6f33961a8aeffc315ff5d4a74c7a39f6142a8a7935508f048474d0ff32992a6d</t>
+          <t>0x9500bf5b6846fee92a67b0c91fbfea74b8f7a29f9e2edf9a22ae104e172317f4</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19527406</t>
+          <t>L19527404</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785415503</t>
+          <t>1785467456</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785693600</t>
+          <t>1785517200</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>58.455115</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,110 +643,774 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>0xdd3c48b46e7e419535742c6600d8d5c0bfbf337cf9d7384d0931d8644057b38b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.0625</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>First League</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha vs FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0x9500bf5b6846fee92a67b0c91fbfea74b8f7a29f9e2edf9a22ae104e172317f4</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19527404</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1785467455</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1785517200</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0x1c93771d6891dfab8458278bde673acf937ec233145cec08e5cbbf6abad22ca4</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.0625</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>First League</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha vs FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0x9500bf5b6846fee92a67b0c91fbfea74b8f7a29f9e2edf9a22ae104e172317f4</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19527404</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1785467402</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1785517200</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0x94f51445b33e0f282b7b2e2a657f02ae3b738ee45fa16dda9267fc320dd63f2e</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.0625</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>First League</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha vs FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0x9500bf5b6846fee92a67b0c91fbfea74b8f7a29f9e2edf9a22ae104e172317f4</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19527404</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1785467401</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1785517200</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>64.0</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0x7a2d2b6948d276131073d7eb95625bb09fee93e0072e6618ec7171f59bef3d9a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.0625</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>First League</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha vs FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0x9500bf5b6846fee92a67b0c91fbfea74b8f7a29f9e2edf9a22ae104e172317f4</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19527404</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1785467400</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1785517200</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0xb45d6395ce739a0bf97a9c585d0c3aa5d6e2da00ec07295407594c566a55e0a5</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.0625</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>First League</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha vs FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0x9500bf5b6846fee92a67b0c91fbfea74b8f7a29f9e2edf9a22ae104e172317f4</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>L19527404</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1785467398</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1785517200</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>0x4449ee9e19610ed1a6459a4ec622295d3b7f27785ad56fb418383aa2562ee601</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0x34FcBC23fB24111d68542f4B3cF185543Af2fA25</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.5987</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>First League</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>FK Pardubice vs FK Jablonec</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>FK Pardubice</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>FK Jablonec</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0x6f33961a8aeffc315ff5d4a74c7a39f6142a8a7935508f048474d0ff32992a6d</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19527406</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1785415503</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1785693600</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>58.455115</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>0x19f2092f5b69321f498e3935667243b7f359a9876c356076e23b9a65276c6308</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>0.99998</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>1.8363</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>AC Sparta Praha</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>First League</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>AC Sparta Praha vs FC Fastav Zlín</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>AC Sparta Praha</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>FC Fastav Zlín</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>0x030b420c1d99e5824e84934cc2cf515e30fa8607adbe9c86574bc07d04d89b58</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>L19527404</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>1785344291</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>1785517200</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>1.195791</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-31 13:04:00 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/First League/trades.xlsx
+++ b/data/sxbet/ligas/First League/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x5826b25b9a78e0be2b5364f99906ff8cc4bf845a562a5ea97f684cd2f19405ae</t>
+          <t>0x750959461898d7985dfb52df9d12bdc41ab62fe003f6662c5f2c1f5e6883c3b3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
+          <t>0xA44AB2Cf43d5D82896598FF80855897B50aC323A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>13.2855</t>
+          <t>15.12</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.07</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1.FC Slovacko</t>
+          <t>FC Fastav Zlín</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.FC Slovacko vs Sk Artis Brno</t>
+          <t>AC Sparta Praha vs FC Fastav Zlín</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1.FC Slovacko</t>
+          <t>AC Sparta Praha</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Sk Artis Brno</t>
+          <t>FC Fastav Zlín</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x10b10a8752de2c6583c0e8fbd3093ad3016bc296293b0a09ba25166e401e636f</t>
+          <t>0x9500bf5b6846fee92a67b0c91fbfea74b8f7a29f9e2edf9a22ae104e172317f4</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19527405</t>
+          <t>L19527404</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785483401</t>
+          <t>1785502250</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785596400</t>
+          <t>1785517200</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>22.1425</t>
+          <t>216.0</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,31 +643,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xe630cfdee3f17d67e170b23665fcaae89fd50d2dc2f339c76f4a1abe7a079fc6</t>
+          <t>0x8f3fc6c2b9b98811247c39740afa1dcc5d19110f7099bc28c5d7d72ac810cac5</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0xA44AB2Cf43d5D82896598FF80855897B50aC323A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>14.025</t>
+          <t>11.61173</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.425</t>
+          <t>1.0713</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>First League</t>
@@ -690,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xaeedc6f6ec1744a71bd9be08dbc5f609f00c2c03449f55bd855097430952e5b5</t>
+          <t>0x9500bf5b6846fee92a67b0c91fbfea74b8f7a29f9e2edf9a22ae104e172317f4</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -720,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785476192</t>
+          <t>1785499628</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>162.971649</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x5743b3baab7d0b4196ffe72f2ea5f72938b9bc8bd6e7156319c249a8e1d4977e</t>
+          <t>0x5826b25b9a78e0be2b5364f99906ff8cc4bf845a562a5ea97f684cd2f19405ae</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -762,12 +770,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>13.2855</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.0625</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -777,7 +785,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>FC Fastav Zlín</t>
+          <t>1.FC Slovacko</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -787,27 +795,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>AC Sparta Praha vs FC Fastav Zlín</t>
+          <t>1.FC Slovacko vs Sk Artis Brno</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>AC Sparta Praha</t>
+          <t>1.FC Slovacko</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>FC Fastav Zlín</t>
+          <t>Sk Artis Brno</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x9500bf5b6846fee92a67b0c91fbfea74b8f7a29f9e2edf9a22ae104e172317f4</t>
+          <t>0x10b10a8752de2c6583c0e8fbd3093ad3016bc296293b0a09ba25166e401e636f</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19527404</t>
+          <t>L19527405</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +840,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785467456</t>
+          <t>1785483401</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785517200</t>
+          <t>1785596400</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>22.1425</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,62 +867,54 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xdd3c48b46e7e419535742c6600d8d5c0bfbf337cf9d7384d0931d8644057b38b</t>
+          <t>0xe630cfdee3f17d67e170b23665fcaae89fd50d2dc2f339c76f4a1abe7a079fc6</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>14.025</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.0625</t>
+          <t>1.425</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>First League</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha vs FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>FC Fastav Zlín</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>First League</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>AC Sparta Praha vs FC Fastav Zlín</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>AC Sparta Praha</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>FC Fastav Zlín</t>
-        </is>
-      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x9500bf5b6846fee92a67b0c91fbfea74b8f7a29f9e2edf9a22ae104e172317f4</t>
+          <t>0xaeedc6f6ec1744a71bd9be08dbc5f609f00c2c03449f55bd855097430952e5b5</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785467455</t>
+          <t>1785476192</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +971,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x1c93771d6891dfab8458278bde673acf937ec233145cec08e5cbbf6abad22ca4</t>
+          <t>0x5743b3baab7d0b4196ffe72f2ea5f72938b9bc8bd6e7156319c249a8e1d4977e</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785467402</t>
+          <t>1785467456</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,7 +1083,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x94f51445b33e0f282b7b2e2a657f02ae3b738ee45fa16dda9267fc320dd63f2e</t>
+          <t>0xdd3c48b46e7e419535742c6600d8d5c0bfbf337cf9d7384d0931d8644057b38b</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785467401</t>
+          <t>1785467455</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,7 +1195,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x7a2d2b6948d276131073d7eb95625bb09fee93e0072e6618ec7171f59bef3d9a</t>
+          <t>0x1c93771d6891dfab8458278bde673acf937ec233145cec08e5cbbf6abad22ca4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785467400</t>
+          <t>1785467402</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xb45d6395ce739a0bf97a9c585d0c3aa5d6e2da00ec07295407594c566a55e0a5</t>
+          <t>0x94f51445b33e0f282b7b2e2a657f02ae3b738ee45fa16dda9267fc320dd63f2e</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785467398</t>
+          <t>1785467401</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1419,23 +1419,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x4449ee9e19610ed1a6459a4ec622295d3b7f27785ad56fb418383aa2562ee601</t>
+          <t>0x7a2d2b6948d276131073d7eb95625bb09fee93e0072e6618ec7171f59bef3d9a</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x34FcBC23fB24111d68542f4B3cF185543Af2fA25</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.5987</t>
+          <t>1.0625</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1443,7 +1447,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>First League</t>
@@ -1451,27 +1459,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>FK Pardubice vs FK Jablonec</t>
+          <t>AC Sparta Praha vs FC Fastav Zlín</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>FK Pardubice</t>
+          <t>AC Sparta Praha</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>FK Jablonec</t>
+          <t>FC Fastav Zlín</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x6f33961a8aeffc315ff5d4a74c7a39f6142a8a7935508f048474d0ff32992a6d</t>
+          <t>0x9500bf5b6846fee92a67b0c91fbfea74b8f7a29f9e2edf9a22ae104e172317f4</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19527406</t>
+          <t>L19527404</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1496,17 +1504,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785415503</t>
+          <t>1785467400</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1785693600</t>
+          <t>1785517200</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>58.455115</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1523,110 +1531,326 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>0xb45d6395ce739a0bf97a9c585d0c3aa5d6e2da00ec07295407594c566a55e0a5</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.0625</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>First League</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha vs FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>FC Fastav Zlín</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0x9500bf5b6846fee92a67b0c91fbfea74b8f7a29f9e2edf9a22ae104e172317f4</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>L19527404</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1785467398</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1785517200</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>0x4449ee9e19610ed1a6459a4ec622295d3b7f27785ad56fb418383aa2562ee601</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0x34FcBC23fB24111d68542f4B3cF185543Af2fA25</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.5987</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>First League</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>FK Pardubice vs FK Jablonec</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>FK Pardubice</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>FK Jablonec</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0x6f33961a8aeffc315ff5d4a74c7a39f6142a8a7935508f048474d0ff32992a6d</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>L19527406</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1785415503</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1785693600</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>58.455115</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>0x19f2092f5b69321f498e3935667243b7f359a9876c356076e23b9a65276c6308</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>0.99998</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>1.8363</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>AC Sparta Praha</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>First League</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>AC Sparta Praha vs FC Fastav Zlín</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>AC Sparta Praha</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>FC Fastav Zlín</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>0x030b420c1d99e5824e84934cc2cf515e30fa8607adbe9c86574bc07d04d89b58</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>L19527404</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
         <is>
           <t>1785344291</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>1785517200</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>1.195791</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>